<commit_message>
Add Hovland ORCID and correct hDRG submission metadata
</commit_message>
<xml_diff>
--- a/sra_submission/Cheng_TGN_BioSample_Human1.0.xlsx
+++ b/sra_submission/Cheng_TGN_BioSample_Human1.0.xlsx
@@ -570,7 +570,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD31"/>
+  <dimension ref="A1:AE31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26.140625" customWidth="1" style="1" min="1" max="1"/>
@@ -829,6 +829,11 @@
           <t>sample_role</t>
         </is>
       </c>
+      <c r="AE12" t="inlineStr">
+        <is>
+          <t>supplier_catalog_number</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -921,6 +926,11 @@
           <t>TGN culture</t>
         </is>
       </c>
+      <c r="AE13" t="inlineStr">
+        <is>
+          <t>not applicable</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1013,6 +1023,11 @@
           <t>TGN culture</t>
         </is>
       </c>
+      <c r="AE14" t="inlineStr">
+        <is>
+          <t>not applicable</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1105,6 +1120,11 @@
           <t>TGN culture</t>
         </is>
       </c>
+      <c r="AE15" t="inlineStr">
+        <is>
+          <t>not applicable</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1197,6 +1217,11 @@
           <t>TGN culture</t>
         </is>
       </c>
+      <c r="AE16" t="inlineStr">
+        <is>
+          <t>not applicable</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1289,6 +1314,11 @@
           <t>TGN culture</t>
         </is>
       </c>
+      <c r="AE17" t="inlineStr">
+        <is>
+          <t>not applicable</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1381,6 +1411,11 @@
           <t>TGN culture</t>
         </is>
       </c>
+      <c r="AE18" t="inlineStr">
+        <is>
+          <t>not applicable</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1473,6 +1508,11 @@
           <t>TGN culture</t>
         </is>
       </c>
+      <c r="AE19" t="inlineStr">
+        <is>
+          <t>not applicable</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1565,6 +1605,11 @@
           <t>TGN culture</t>
         </is>
       </c>
+      <c r="AE20" t="inlineStr">
+        <is>
+          <t>not applicable</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1657,6 +1702,11 @@
           <t>TGN culture</t>
         </is>
       </c>
+      <c r="AE21" t="inlineStr">
+        <is>
+          <t>not applicable</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1749,6 +1799,11 @@
           <t>TGN culture</t>
         </is>
       </c>
+      <c r="AE22" t="inlineStr">
+        <is>
+          <t>not applicable</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1841,6 +1896,11 @@
           <t>TGN culture</t>
         </is>
       </c>
+      <c r="AE23" t="inlineStr">
+        <is>
+          <t>not applicable</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1933,6 +1993,11 @@
           <t>TGN culture</t>
         </is>
       </c>
+      <c r="AE24" t="inlineStr">
+        <is>
+          <t>not applicable</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2025,6 +2090,11 @@
           <t>TGN culture</t>
         </is>
       </c>
+      <c r="AE25" t="inlineStr">
+        <is>
+          <t>not applicable</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2089,7 +2159,7 @@
       </c>
       <c r="AA26" t="inlineStr">
         <is>
-          <t>Commercial pooled human dorsal root ganglion RNA from Takara Bio; source pool 1 comprises 21 donors; C1 and C2 are technical sequencing runs.</t>
+          <t>Commercial pooled human dorsal root ganglion RNA from Takara Bio, Cat# 636150; source lot 1 is described in the manuscript as pooled from 21 normal donors aged 16-65 years; C1 and C2 are technical sequencing runs.</t>
         </is>
       </c>
       <c r="AB26" t="inlineStr">
@@ -2105,6 +2175,11 @@
       <c r="AD26" t="inlineStr">
         <is>
           <t>hDRG comparator 1</t>
+        </is>
+      </c>
+      <c r="AE26" t="inlineStr">
+        <is>
+          <t>636150</t>
         </is>
       </c>
     </row>
@@ -2131,7 +2206,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>not collected</t>
+          <t>16-65 years</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -2151,7 +2226,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>not collected</t>
+          <t>not applicable</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2159,6 +2234,11 @@
           <t>dorsal root ganglion</t>
         </is>
       </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
       <c r="Y27" t="inlineStr">
         <is>
           <t>tissue sample</t>
@@ -2166,7 +2246,7 @@
       </c>
       <c r="AA27" t="inlineStr">
         <is>
-          <t>Second, separate pool of commercial human dorsal root ganglion RNA from Takara Bio; C1 and C2 are technical sequencing runs of this pool.</t>
+          <t>Second, separate lot of commercial pooled human dorsal root ganglion RNA from Takara Bio, Cat# 636150; the manuscript describes the two lots as from 21 normal donors aged 16-65 years; C1 and C2 are technical sequencing runs of this lot.</t>
         </is>
       </c>
       <c r="AB27" t="inlineStr">
@@ -2182,6 +2262,11 @@
       <c r="AD27" t="inlineStr">
         <is>
           <t>hDRG comparator 2</t>
+        </is>
+      </c>
+      <c r="AE27" t="inlineStr">
+        <is>
+          <t>636150</t>
         </is>
       </c>
     </row>

</xml_diff>